<commit_message>
update relatorio_anuncios.xlsx: modify radio capture report file
</commit_message>
<xml_diff>
--- a/radio_capture/relatorio_anuncios.xlsx
+++ b/radio_capture/relatorio_anuncios.xlsx
@@ -42,7 +42,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -303,6 +308,24 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -673,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -723,27 +746,27 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="67" t="inlineStr">
+      <c r="A2" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:00:14</t>
         </is>
       </c>
-      <c r="B2" s="67" t="inlineStr">
+      <c r="B2" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C2" s="67" t="inlineStr">
+      <c r="C2" s="72" t="inlineStr">
         <is>
           <t>Casa dos Construtores</t>
         </is>
       </c>
-      <c r="D2" s="67" t="inlineStr">
+      <c r="D2" s="72" t="inlineStr">
         <is>
           <t>espaços para casas</t>
         </is>
       </c>
-      <c r="E2" s="67" t="inlineStr">
+      <c r="E2" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -753,34 +776,34 @@
           <t>Mas em como se vive? O tempo bem vivido é feito de escolhas, de detalhes que permanecem, de casas que acolhem, de memórias que resistem. Há 65 anos, criamos espaços para que cada instante não apenas p</t>
         </is>
       </c>
-      <c r="G2" s="67" t="inlineStr">
+      <c r="G2" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Casa_dos_Construtores__espacos_para_casas__09-03-2026_09-00-14__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="67" t="inlineStr">
+      <c r="A3" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:00:15</t>
         </is>
       </c>
-      <c r="B3" s="67" t="inlineStr">
+      <c r="B3" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C3" s="67" t="inlineStr">
+      <c r="C3" s="72" t="inlineStr">
         <is>
           <t>Ótica Fabriley</t>
         </is>
       </c>
-      <c r="D3" s="67" t="inlineStr">
+      <c r="D3" s="72" t="inlineStr">
         <is>
           <t>serviços de ótica</t>
         </is>
       </c>
-      <c r="E3" s="67" t="inlineStr">
+      <c r="E3" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -790,34 +813,34 @@
           <t>Mas em como se vive? O tempo bem vivido é feito de escolhas, de detalhes que permanecem, de casas que acolhem, de memórias que resistem. Há 65 anos, criamos espaços para que cada instante não apenas p</t>
         </is>
       </c>
-      <c r="G3" s="67" t="inlineStr">
+      <c r="G3" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Otica_Fabriley__servicos_de_otica__09-03-2026_09-00-15__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="67" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:00:31</t>
         </is>
       </c>
-      <c r="B4" s="67" t="inlineStr">
+      <c r="B4" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C4" s="67" t="inlineStr">
+      <c r="C4" s="72" t="inlineStr">
         <is>
           <t>ótica FabriLen</t>
         </is>
       </c>
-      <c r="D4" s="67" t="inlineStr">
+      <c r="D4" s="72" t="inlineStr">
         <is>
           <t>lentes</t>
         </is>
       </c>
-      <c r="E4" s="67" t="inlineStr">
+      <c r="E4" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -827,34 +850,34 @@
           <t>Cada instante, não apenas passe, mas fique. Casa dos Construtores, o melhor tempo na sua casa. Quando o assunto é visão, a ótica FabriLen é referência. Atendimento diferenciado com profissionais prepa</t>
         </is>
       </c>
-      <c r="G4" s="67" t="inlineStr">
+      <c r="G4" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__otica_FabriLen__lentes__09-03-2026_09-00-30.mp3</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="67" t="inlineStr">
+      <c r="A5" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:00:33</t>
         </is>
       </c>
-      <c r="B5" s="67" t="inlineStr">
+      <c r="B5" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C5" s="67" t="inlineStr">
+      <c r="C5" s="72" t="inlineStr">
         <is>
           <t>Cacau Show</t>
         </is>
       </c>
-      <c r="D5" s="67" t="inlineStr">
+      <c r="D5" s="72" t="inlineStr">
         <is>
           <t>Chocolate</t>
         </is>
       </c>
-      <c r="E5" s="67" t="inlineStr">
+      <c r="E5" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -864,34 +887,34 @@
           <t>Viu? Bob Sinclair na programação número 1 do seu rádio, vocês viram aí, aliás, ouviram, né? Vai, Tassonzão! Tonsera, né, pra gente curtir aqui na programação. Jovem Pan, daqui a pouquinho, depois de i</t>
         </is>
       </c>
-      <c r="G5" s="67" t="inlineStr">
+      <c r="G5" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Cacau_Show__Chocolate__09-03-2026_09-00-33.mp3</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="67" t="inlineStr">
+      <c r="A6" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:00:48</t>
         </is>
       </c>
-      <c r="B6" s="67" t="inlineStr">
+      <c r="B6" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C6" s="67" t="inlineStr">
+      <c r="C6" s="72" t="inlineStr">
         <is>
           <t>Noblen</t>
         </is>
       </c>
-      <c r="D6" s="67" t="inlineStr">
+      <c r="D6" s="72" t="inlineStr">
         <is>
           <t>lentes multifocais digitais e lentes de visão simples</t>
         </is>
       </c>
-      <c r="E6" s="67" t="inlineStr">
+      <c r="E6" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -901,34 +924,34 @@
           <t>Preparados para orientar você com atenção e confiança. As lentes são produzidas com alta tecnologia, garantindo precisão e conforto para o dia a dia. E tem promoção especial. Na compra do primeiro par</t>
         </is>
       </c>
-      <c r="G6" s="67" t="inlineStr">
+      <c r="G6" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Noblen__lentes_multifocais_digitais_e_lentes_de_visao_simples__09-03-2026_09-00-48.mp3</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="67" t="inlineStr">
+      <c r="A7" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:00:50</t>
         </is>
       </c>
-      <c r="B7" s="67" t="inlineStr">
+      <c r="B7" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C7" s="67" t="inlineStr">
+      <c r="C7" s="72" t="inlineStr">
         <is>
           <t>Cacau Show</t>
         </is>
       </c>
-      <c r="D7" s="67" t="inlineStr">
+      <c r="D7" s="72" t="inlineStr">
         <is>
           <t>chocolate</t>
         </is>
       </c>
-      <c r="E7" s="67" t="inlineStr">
+      <c r="E7" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -938,34 +961,34 @@
           <t>Número 1 do Brasil e... e... e... Cacau Show! Aquele chocolate maravilhoso, aquele chocolate refinado, aquele sabor... Hummm... já vai dando assim o negócio, é de louco, né? Quer levar pra casa? Então</t>
         </is>
       </c>
-      <c r="G7" s="67" t="inlineStr">
+      <c r="G7" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Cacau_Show__chocolate__09-03-2026_09-00-50.mp3</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="67" t="inlineStr">
+      <c r="A8" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:01:04</t>
         </is>
       </c>
-      <c r="B8" s="67" t="inlineStr">
+      <c r="B8" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C8" s="67" t="inlineStr">
+      <c r="C8" s="72" t="inlineStr">
         <is>
           <t>Óticas FabriLem</t>
         </is>
       </c>
-      <c r="D8" s="67" t="inlineStr">
+      <c r="D8" s="72" t="inlineStr">
         <is>
           <t>lentes de visão simples com antirreflexo e filtro de luz azul</t>
         </is>
       </c>
-      <c r="E8" s="67" t="inlineStr">
+      <c r="E8" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -975,7 +998,7 @@
           <t>digitais noblem com antirreflexo, o segundo par é grátis. E mais, lentes de visão simples com antirreflexo e filtro de luz azul em até dez vezes de dezoito e noventa. Visite a loja na Rua Brasil Esqui</t>
         </is>
       </c>
-      <c r="G8" s="67" t="inlineStr">
+      <c r="G8" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Oticas_FabriLem__lentes_de_visao_simples_com_antirreflexo_e_filtro_de_luz_azu__09-03-2026_09-01-04__ad1.mp3</t>
         </is>
@@ -1019,27 +1042,27 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="67" t="inlineStr">
+      <c r="A10" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:01:21</t>
         </is>
       </c>
-      <c r="B10" s="67" t="inlineStr">
+      <c r="B10" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C10" s="67" t="inlineStr">
+      <c r="C10" s="72" t="inlineStr">
         <is>
           <t>Amaral Centro Automotivo Multimarcas</t>
         </is>
       </c>
-      <c r="D10" s="67" t="inlineStr">
+      <c r="D10" s="72" t="inlineStr">
         <is>
           <t>serviços automotivos</t>
         </is>
       </c>
-      <c r="E10" s="67" t="inlineStr">
+      <c r="E10" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1049,34 +1072,34 @@
           <t>FabriLem, a fábrica da sua lente. Amaral Centro Automotivo Multimarcas agradece a todos o carinho e a confiança no trabalho realizado com sua equipe de profissionais. Hoje estamos em novo endereço par</t>
         </is>
       </c>
-      <c r="G10" s="67" t="inlineStr">
+      <c r="G10" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Amaral_Centro_Automotivo_Multimarcas__servicos_automotivos__09-03-2026_09-01-21.mp3</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="67" t="inlineStr">
+      <c r="A11" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:02:10</t>
         </is>
       </c>
-      <c r="B11" s="67" t="inlineStr">
+      <c r="B11" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C11" s="67" t="inlineStr">
+      <c r="C11" s="72" t="inlineStr">
         <is>
           <t>Unifipa</t>
         </is>
       </c>
-      <c r="D11" s="67" t="inlineStr">
+      <c r="D11" s="72" t="inlineStr">
         <is>
           <t>Cursos de graduação</t>
         </is>
       </c>
-      <c r="E11" s="67" t="inlineStr">
+      <c r="E11" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1086,7 +1109,7 @@
           <t>São onze opções de cursos de graduação na instituição que tem mais de cinquenta e cinco anos de tradição e é sinônimo de excelência em ensino com nota máxima na avaliação do MEC. Venha ser Unifipa. In</t>
         </is>
       </c>
-      <c r="G11" s="67" t="inlineStr">
+      <c r="G11" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Unifipa__Cursos_de_graduacao__09-03-2026_09-02-10__ad1.mp3</t>
         </is>
@@ -1130,27 +1153,27 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="67" t="inlineStr">
+      <c r="A13" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:02:27</t>
         </is>
       </c>
-      <c r="B13" s="67" t="inlineStr">
+      <c r="B13" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C13" s="67" t="inlineStr">
+      <c r="C13" s="72" t="inlineStr">
         <is>
           <t>Cicred</t>
         </is>
       </c>
-      <c r="D13" s="67" t="inlineStr">
+      <c r="D13" s="72" t="inlineStr">
         <is>
           <t>Poupança premiada</t>
         </is>
       </c>
-      <c r="E13" s="67" t="inlineStr">
+      <c r="E13" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1160,34 +1183,34 @@
           <t>A Unipipa, referência que transforma vidas. Aqui é a Nagacela, é hora de sonhar alto. A poupança premiada Cicred tá aí. Cicred, poupança é premiada Pra fazer tudo o que você sonhava Tem milhões em ben</t>
         </is>
       </c>
-      <c r="G13" s="67" t="inlineStr">
+      <c r="G13" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Cicred__Poupanca_premiada__09-03-2026_09-02-27.mp3</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="67" t="inlineStr">
+      <c r="A14" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:02:43</t>
         </is>
       </c>
-      <c r="B14" s="67" t="inlineStr">
+      <c r="B14" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C14" s="67" t="inlineStr">
+      <c r="C14" s="72" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="D14" s="67" t="inlineStr">
+      <c r="D14" s="72" t="inlineStr">
         <is>
           <t>Produtos para Páscoa (chocolate, ovo de Páscoa, peixe, etc.)</t>
         </is>
       </c>
-      <c r="E14" s="67" t="inlineStr">
+      <c r="E14" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1197,34 +1220,34 @@
           <t>São mais de 600 ganhadores, 5 milhões em prêmios em dinheiro. Volte no Cicred e concorra! O Baré Show, olha onde eu tô! Corre para conferir os preços imperdíveis do Max e garanta sua Páscoa! Olha, tem</t>
         </is>
       </c>
-      <c r="G14" s="67" t="inlineStr">
+      <c r="G14" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Max__Produtos_para_Pascoa__chocolate__ovo_de_Pascoa__peixe__etc__09-03-2026_09-02-43__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="67" t="inlineStr">
+      <c r="A15" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:02:43</t>
         </is>
       </c>
-      <c r="B15" s="67" t="inlineStr">
+      <c r="B15" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C15" s="67" t="inlineStr">
+      <c r="C15" s="72" t="inlineStr">
         <is>
           <t>Cicred</t>
         </is>
       </c>
-      <c r="D15" s="67" t="inlineStr">
+      <c r="D15" s="72" t="inlineStr">
         <is>
           <t>Concurso com prêmios em dinheiro</t>
         </is>
       </c>
-      <c r="E15" s="67" t="inlineStr">
+      <c r="E15" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1234,34 +1257,34 @@
           <t>São mais de 600 ganhadores, 5 milhões em prêmios em dinheiro. Volte no Cicred e concorra! O Baré Show, olha onde eu tô! Corre para conferir os preços imperdíveis do Max e garanta sua Páscoa! Olha, tem</t>
         </is>
       </c>
-      <c r="G15" s="67" t="inlineStr">
+      <c r="G15" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Cicred__Concurso_com_premios_em_dinheiro__09-03-2026_09-02-43__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="67" t="inlineStr">
+      <c r="A16" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:00</t>
         </is>
       </c>
-      <c r="B16" s="67" t="inlineStr">
+      <c r="B16" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C16" s="67" t="inlineStr">
+      <c r="C16" s="72" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="D16" s="67" t="inlineStr">
+      <c r="D16" s="72" t="inlineStr">
         <is>
           <t>Produtos para Páscoa (chocolate, ovo de Páscoa, peixe, etc.)</t>
         </is>
       </c>
-      <c r="E16" s="67" t="inlineStr">
+      <c r="E16" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1271,34 +1294,34 @@
           <t>Corre para conferir os preços imperdíveis do Max e garanta sua Páscoa. Olha, tem chocolate, ovo de Páscoa, peixe e muito mais. Tudo com preço baixinho pra você aproveitar. Filé de peito lá no quilo 14</t>
         </is>
       </c>
-      <c r="G16" s="67" t="inlineStr">
+      <c r="G16" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Max__Produtos_para_Pascoa__chocolate__ovo_de_Pascoa__peixe__etc__09-03-2026_09-03-00.mp3</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="67" t="inlineStr">
+      <c r="A17" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:14</t>
         </is>
       </c>
-      <c r="B17" s="67" t="inlineStr">
+      <c r="B17" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C17" s="67" t="inlineStr">
+      <c r="C17" s="72" t="inlineStr">
         <is>
           <t>Netflix</t>
         </is>
       </c>
-      <c r="D17" s="67" t="inlineStr">
+      <c r="D17" s="72" t="inlineStr">
         <is>
           <t>BTS The Comeback Live</t>
         </is>
       </c>
-      <c r="E17" s="67" t="inlineStr">
+      <c r="E17" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1308,34 +1331,34 @@
           <t xml:space="preserve">Uma delas é o trailer do especial da Netflix, BTS The Comeback Live, que chega à plataforma no próximo dia 20. O filme faz parte da poderosa campanha promocional do álbum I Run dos reis do K-Pop. Pra </t>
         </is>
       </c>
-      <c r="G17" s="67" t="inlineStr">
+      <c r="G17" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Netflix__BTS_The_Comeback_Live__09-03-2026_09-03-14.mp3</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="67" t="inlineStr">
+      <c r="A18" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:16</t>
         </is>
       </c>
-      <c r="B18" s="67" t="inlineStr">
+      <c r="B18" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C18" s="67" t="inlineStr">
+      <c r="C18" s="72" t="inlineStr">
         <is>
           <t>Sete Farinha Globo</t>
         </is>
       </c>
-      <c r="D18" s="67" t="inlineStr">
+      <c r="D18" s="72" t="inlineStr">
         <is>
           <t>Farinha</t>
         </is>
       </c>
-      <c r="E18" s="67" t="inlineStr">
+      <c r="E18" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1345,34 +1368,34 @@
           <t>sete farinha globo, um quilo, dois e quarenta e sete. Tó de trezentos e setenta gramas, sete e noventa e nove. Mussarela a partir de vinte e seis e noventa um quilo. Papel Supra, vinte e nove e novent</t>
         </is>
       </c>
-      <c r="G18" s="67" t="inlineStr">
+      <c r="G18" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Sete_Farinha_Globo__Farinha__09-03-2026_09-03-16__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="67" t="inlineStr">
+      <c r="A19" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:16</t>
         </is>
       </c>
-      <c r="B19" s="67" t="inlineStr">
+      <c r="B19" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C19" s="67" t="inlineStr">
+      <c r="C19" s="72" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="D19" s="67" t="inlineStr">
+      <c r="D19" s="72" t="inlineStr">
         <is>
           <t>Pasta</t>
         </is>
       </c>
-      <c r="E19" s="67" t="inlineStr">
+      <c r="E19" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1382,34 +1405,34 @@
           <t>sete farinha globo, um quilo, dois e quarenta e sete. Tó de trezentos e setenta gramas, sete e noventa e nove. Mussarela a partir de vinte e seis e noventa um quilo. Papel Supra, vinte e nove e novent</t>
         </is>
       </c>
-      <c r="G19" s="67" t="inlineStr">
+      <c r="G19" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Max__Pasta__09-03-2026_09-03-16__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="67" t="inlineStr">
+      <c r="A20" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:16</t>
         </is>
       </c>
-      <c r="B20" s="67" t="inlineStr">
+      <c r="B20" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C20" s="67" t="inlineStr">
+      <c r="C20" s="72" t="inlineStr">
         <is>
           <t>Drogaria Total Popular</t>
         </is>
       </c>
-      <c r="D20" s="67" t="inlineStr">
+      <c r="D20" s="72" t="inlineStr">
         <is>
           <t>Remédios</t>
         </is>
       </c>
-      <c r="E20" s="67" t="inlineStr">
+      <c r="E20" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1419,34 +1442,34 @@
           <t>sete farinha globo, um quilo, dois e quarenta e sete. Tó de trezentos e setenta gramas, sete e noventa e nove. Mussarela a partir de vinte e seis e noventa um quilo. Papel Supra, vinte e nove e novent</t>
         </is>
       </c>
-      <c r="G20" s="67" t="inlineStr">
+      <c r="G20" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Drogaria_Total_Popular__Remedios__09-03-2026_09-03-16__ad3.mp3</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="67" t="inlineStr">
+      <c r="A21" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:32</t>
         </is>
       </c>
-      <c r="B21" s="67" t="inlineStr">
+      <c r="B21" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C21" s="67" t="inlineStr">
+      <c r="C21" s="72" t="inlineStr">
         <is>
           <t>Doutor Alex Baraldo Portes</t>
         </is>
       </c>
-      <c r="D21" s="67" t="inlineStr">
+      <c r="D21" s="72" t="inlineStr">
         <is>
           <t>Serviços de Otorrino Laringologista</t>
         </is>
       </c>
-      <c r="E21" s="67" t="inlineStr">
+      <c r="E21" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1456,34 +1479,34 @@
           <t xml:space="preserve">Jovem Pan. Jovem Pan Brasil. Você está ouvindo. Manhã Pan. Catanduva. Oferecimento. Doutor Alex Baraldo Portes. Otorrino Laringologista. RQE 64202. Vive em empreendimentos. Municipa Catanduva. Doutor </t>
         </is>
       </c>
-      <c r="G21" s="67" t="inlineStr">
+      <c r="G21" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Doutor_Alex_Baraldo_Portes__Servicos_de_Otorrino_Laringologista__09-03-2026_09-03-32__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="67" t="inlineStr">
+      <c r="A22" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:32</t>
         </is>
       </c>
-      <c r="B22" s="67" t="inlineStr">
+      <c r="B22" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C22" s="67" t="inlineStr">
+      <c r="C22" s="72" t="inlineStr">
         <is>
           <t>IGA Proteção Veicular</t>
         </is>
       </c>
-      <c r="D22" s="67" t="inlineStr">
+      <c r="D22" s="72" t="inlineStr">
         <is>
           <t>Proteção Veicular</t>
         </is>
       </c>
-      <c r="E22" s="67" t="inlineStr">
+      <c r="E22" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1493,34 +1516,34 @@
           <t xml:space="preserve">Jovem Pan. Jovem Pan Brasil. Você está ouvindo. Manhã Pan. Catanduva. Oferecimento. Doutor Alex Baraldo Portes. Otorrino Laringologista. RQE 64202. Vive em empreendimentos. Municipa Catanduva. Doutor </t>
         </is>
       </c>
-      <c r="G22" s="67" t="inlineStr">
+      <c r="G22" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__IGA_Protecao_Veicular__Protecao_Veicular__09-03-2026_09-03-32__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="67" t="inlineStr">
+      <c r="A23" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:03:50</t>
         </is>
       </c>
-      <c r="B23" s="67" t="inlineStr">
+      <c r="B23" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C23" s="67" t="inlineStr">
+      <c r="C23" s="72" t="inlineStr">
         <is>
           <t>Doutor Alex Baraldo Portes</t>
         </is>
       </c>
-      <c r="D23" s="67" t="inlineStr">
+      <c r="D23" s="72" t="inlineStr">
         <is>
           <t>Serviços de otorrino laringologista</t>
         </is>
       </c>
-      <c r="E23" s="67" t="inlineStr">
+      <c r="E23" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1530,34 +1553,34 @@
           <t>Municipal, município de Catanduva, doutor Cristiano Herrera e GA Proteção Veicular. Nariz entupido, incômodos no ouvido, nariz ou garganta? Sua saúde pode estar precisando de atenção. Quando você sent</t>
         </is>
       </c>
-      <c r="G23" s="67" t="inlineStr">
+      <c r="G23" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Doutor_Alex_Baraldo_Portes__Servicos_de_otorrino_laringologista__09-03-2026_09-03-50.mp3</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="67" t="inlineStr">
+      <c r="A24" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:04:08</t>
         </is>
       </c>
-      <c r="B24" s="67" t="inlineStr">
+      <c r="B24" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C24" s="67" t="inlineStr">
+      <c r="C24" s="72" t="inlineStr">
         <is>
           <t>Doutor Alex Baraldo Portes</t>
         </is>
       </c>
-      <c r="D24" s="67" t="inlineStr">
+      <c r="D24" s="72" t="inlineStr">
         <is>
           <t>Serviços de otorrino-laringologia</t>
         </is>
       </c>
-      <c r="E24" s="67" t="inlineStr">
+      <c r="E24" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1567,34 +1590,34 @@
           <t>Cuida do nariz, ouvido e garganta. Não perca o foco da sua saúde. Essa é uma mensagem do doutor Alex Baraldo Portes, que é otorrino-laringologista. CRM 137582, RQE 64202. Lá no Instagram do doutor Ale</t>
         </is>
       </c>
-      <c r="G24" s="67" t="inlineStr">
+      <c r="G24" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Doutor_Alex_Baraldo_Portes__Servicos_de_otorrino-laringologia__09-03-2026_09-04-08__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="67" t="inlineStr">
+      <c r="A25" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:04:08</t>
         </is>
       </c>
-      <c r="B25" s="67" t="inlineStr">
+      <c r="B25" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C25" s="67" t="inlineStr">
+      <c r="C25" s="72" t="inlineStr">
         <is>
           <t>Unifipa Catanduva</t>
         </is>
       </c>
-      <c r="D25" s="67" t="inlineStr">
+      <c r="D25" s="72" t="inlineStr">
         <is>
           <t>Vestibular continuado 2026</t>
         </is>
       </c>
-      <c r="E25" s="67" t="inlineStr">
+      <c r="E25" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1604,34 +1627,34 @@
           <t>Cuida do nariz, ouvido e garganta. Não perca o foco da sua saúde. Essa é uma mensagem do doutor Alex Baraldo Portes, que é otorrino-laringologista. CRM 137582, RQE 64202. Lá no Instagram do doutor Ale</t>
         </is>
       </c>
-      <c r="G25" s="67" t="inlineStr">
+      <c r="G25" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Unifipa_Catanduva__Vestibular_continuado_2026__09-03-2026_09-04-08__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="67" t="inlineStr">
+      <c r="A26" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:04:22</t>
         </is>
       </c>
-      <c r="B26" s="67" t="inlineStr">
+      <c r="B26" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C26" s="67" t="inlineStr">
+      <c r="C26" s="72" t="inlineStr">
         <is>
           <t>Netflix</t>
         </is>
       </c>
-      <c r="D26" s="67" t="inlineStr">
+      <c r="D26" s="72" t="inlineStr">
         <is>
           <t>Serviço de streaming</t>
         </is>
       </c>
-      <c r="E26" s="67" t="inlineStr">
+      <c r="E26" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1641,34 +1664,34 @@
           <t>Ligue agora ou mande um zap, dezessete três um cinco um mil, ou acesse NetflixBR.com. É Netflix! A FM da gente, Ondas Verde! A sua manhã fica completa na Ondas Verdes.</t>
         </is>
       </c>
-      <c r="G26" s="67" t="inlineStr">
+      <c r="G26" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Netflix__Servico_de_streaming__09-03-2026_09-04-22.mp3</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="67" t="inlineStr">
+      <c r="A27" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:04:44</t>
         </is>
       </c>
-      <c r="B27" s="67" t="inlineStr">
+      <c r="B27" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C27" s="67" t="inlineStr">
+      <c r="C27" s="72" t="inlineStr">
         <is>
           <t>Unifipa</t>
         </is>
       </c>
-      <c r="D27" s="67" t="inlineStr">
+      <c r="D27" s="72" t="inlineStr">
         <is>
           <t>Inscrições e provas online</t>
         </is>
       </c>
-      <c r="E27" s="67" t="inlineStr">
+      <c r="E27" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1678,34 +1701,34 @@
           <t>é que venha ser Unifipa, inscrições e provas online em unifipa.com.br barra vestibular. Unifipa, referência que transforma vidas. A clínica do doutor Cristiano Herrera, gente, atenção, é referência na</t>
         </is>
       </c>
-      <c r="G27" s="67" t="inlineStr">
+      <c r="G27" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Unifipa__Inscricoes_e_provas_online__09-03-2026_09-04-44__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="67" t="inlineStr">
+      <c r="A28" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:04:45</t>
         </is>
       </c>
-      <c r="B28" s="67" t="inlineStr">
+      <c r="B28" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C28" s="67" t="inlineStr">
+      <c r="C28" s="72" t="inlineStr">
         <is>
           <t>Clínica do Doutor Cristiano Herrera</t>
         </is>
       </c>
-      <c r="D28" s="67" t="inlineStr">
+      <c r="D28" s="72" t="inlineStr">
         <is>
           <t>Serviços de psicologia, neuropsicologia e psicopedagogia</t>
         </is>
       </c>
-      <c r="E28" s="67" t="inlineStr">
+      <c r="E28" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1715,34 +1738,34 @@
           <t>é que venha ser Unifipa, inscrições e provas online em unifipa.com.br barra vestibular. Unifipa, referência que transforma vidas. A clínica do doutor Cristiano Herrera, gente, atenção, é referência na</t>
         </is>
       </c>
-      <c r="G28" s="67" t="inlineStr">
+      <c r="G28" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Clinica_do_Doutor_Cristiano_Herrera__Servicos_de_psicologia__neuropsicologia_e_psicopedagogia__09-03-2026_09-04-45__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="67" t="inlineStr">
+      <c r="A29" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:05:02</t>
         </is>
       </c>
-      <c r="B29" s="67" t="inlineStr">
+      <c r="B29" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C29" s="67" t="inlineStr">
+      <c r="C29" s="72" t="inlineStr">
         <is>
           <t>Doutor Cristiano Herrera</t>
         </is>
       </c>
-      <c r="D29" s="67" t="inlineStr">
+      <c r="D29" s="72" t="inlineStr">
         <is>
           <t>Serviços de psicopedagogia e neuropsicologia</t>
         </is>
       </c>
-      <c r="E29" s="67" t="inlineStr">
+      <c r="E29" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1752,34 +1775,34 @@
           <t>Psicopedagogia, através da avaliação neuropsicológica com a equipe multidisciplinar, que você vai encontrar lá, pessoal maravilhoso, o doutor Cristiano Herrera, ele utiliza testes em escalas mais efet</t>
         </is>
       </c>
-      <c r="G29" s="67" t="inlineStr">
+      <c r="G29" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Doutor_Cristiano_Herrera__Servicos_de_psicopedagogia_e_neuropsicologia__09-03-2026_09-05-02__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="67" t="inlineStr">
+      <c r="A30" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:05:03</t>
         </is>
       </c>
-      <c r="B30" s="67" t="inlineStr">
+      <c r="B30" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C30" s="67" t="inlineStr">
+      <c r="C30" s="72" t="inlineStr">
         <is>
           <t>Doutor Cristian Aranjeira</t>
         </is>
       </c>
-      <c r="D30" s="67" t="inlineStr">
+      <c r="D30" s="72" t="inlineStr">
         <is>
           <t>Serviços de psicologia e neuropsicologia</t>
         </is>
       </c>
-      <c r="E30" s="67" t="inlineStr">
+      <c r="E30" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1789,34 +1812,34 @@
           <t>Psicopedagogia, através da avaliação neuropsicológica com a equipe multidisciplinar, que você vai encontrar lá, pessoal maravilhoso, o doutor Cristiano Herrera, ele utiliza testes em escalas mais efet</t>
         </is>
       </c>
-      <c r="G30" s="67" t="inlineStr">
+      <c r="G30" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Doutor_Cristian_Aranjeira__Servicos_de_psicologia_e_neuropsicologia__09-03-2026_09-05-03__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="67" t="inlineStr">
+      <c r="A31" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:05:21</t>
         </is>
       </c>
-      <c r="B31" s="67" t="inlineStr">
+      <c r="B31" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C31" s="67" t="inlineStr">
+      <c r="C31" s="72" t="inlineStr">
         <is>
           <t>Clínica do Dr. Cristiano Herrera</t>
         </is>
       </c>
-      <c r="D31" s="67" t="inlineStr">
+      <c r="D31" s="72" t="inlineStr">
         <is>
           <t>Serviços de psicologia e neuroreabilitação</t>
         </is>
       </c>
-      <c r="E31" s="67" t="inlineStr">
+      <c r="E31" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1826,34 +1849,34 @@
           <t>inclusive os tratamentos não medicamentosos, por exemplo, como neuromodulação e biofeedback. O doutor Cristiano Herrera, ele é psicólogo, neuropsicólogo formado pela USP, especialista em neuroreabilit</t>
         </is>
       </c>
-      <c r="G31" s="67" t="inlineStr">
+      <c r="G31" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Clinica_do_Dr__Cristiano_Herrera__Servicos_de_psicologia_e_neuroreabilitacao__09-03-2026_09-05-21.mp3</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="67" t="inlineStr">
+      <c r="A32" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:05:39</t>
         </is>
       </c>
-      <c r="B32" s="67" t="inlineStr">
+      <c r="B32" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C32" s="67" t="inlineStr">
+      <c r="C32" s="72" t="inlineStr">
         <is>
           <t>Antunes Mais</t>
         </is>
       </c>
-      <c r="D32" s="67" t="inlineStr">
+      <c r="D32" s="72" t="inlineStr">
         <is>
           <t>Arroz seleto e feijão carioca</t>
         </is>
       </c>
-      <c r="E32" s="67" t="inlineStr">
+      <c r="E32" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1863,34 +1886,34 @@
           <t xml:space="preserve">O segundo andar, então acesse arroba DR Cristiano Herrera no Instagram. Liga a fã no Instagram, arroba jovem fã Catanduba. Comece a semana com mais economia no Antunes Mais. Confira arroz seleto tipo </t>
         </is>
       </c>
-      <c r="G32" s="67" t="inlineStr">
+      <c r="G32" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Antunes_Mais__Arroz_seleto_e_feijao_carioca__09-03-2026_09-05-39__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="67" t="inlineStr">
+      <c r="A33" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:05:39</t>
         </is>
       </c>
-      <c r="B33" s="67" t="inlineStr">
+      <c r="B33" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C33" s="67" t="inlineStr">
+      <c r="C33" s="72" t="inlineStr">
         <is>
           <t>Clube do Precinho</t>
         </is>
       </c>
-      <c r="D33" s="67" t="inlineStr">
+      <c r="D33" s="72" t="inlineStr">
         <is>
           <t>Músculo bovino e cortes de carne</t>
         </is>
       </c>
-      <c r="E33" s="67" t="inlineStr">
+      <c r="E33" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1900,34 +1923,34 @@
           <t xml:space="preserve">O segundo andar, então acesse arroba DR Cristiano Herrera no Instagram. Liga a fã no Instagram, arroba jovem fã Catanduba. Comece a semana com mais economia no Antunes Mais. Confira arroz seleto tipo </t>
         </is>
       </c>
-      <c r="G33" s="67" t="inlineStr">
+      <c r="G33" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Clube_do_Precinho__Musculo_bovino_e_cortes_de_carne__09-03-2026_09-05-39__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="67" t="inlineStr">
+      <c r="A34" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:05:57</t>
         </is>
       </c>
-      <c r="B34" s="67" t="inlineStr">
+      <c r="B34" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C34" s="67" t="inlineStr">
+      <c r="C34" s="72" t="inlineStr">
         <is>
           <t>Antunes Mais</t>
         </is>
       </c>
-      <c r="D34" s="67" t="inlineStr">
+      <c r="D34" s="72" t="inlineStr">
         <is>
           <t>Produtos variados (feijão, carne, detergente, etc.)</t>
         </is>
       </c>
-      <c r="E34" s="67" t="inlineStr">
+      <c r="E34" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1937,34 +1960,34 @@
           <t>onze e noventa e nove, feijão carioca seleto, pacote um quilo, seis e noventa e nove, tem também as ofertas do Clube do Precinho, acenho, músculo bovino, trinta e quatro e noventa e cinco quilo, colch</t>
         </is>
       </c>
-      <c r="G34" s="67" t="inlineStr">
+      <c r="G34" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Antunes_Mais__Produtos_variados__feijao__carne__detergente__etc__09-03-2026_09-05-57.mp3</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="67" t="inlineStr">
+      <c r="A35" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:06:15</t>
         </is>
       </c>
-      <c r="B35" s="67" t="inlineStr">
+      <c r="B35" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C35" s="67" t="inlineStr">
+      <c r="C35" s="72" t="inlineStr">
         <is>
           <t>Antunes Mais</t>
         </is>
       </c>
-      <c r="D35" s="67" t="inlineStr">
+      <c r="D35" s="72" t="inlineStr">
         <is>
           <t>Produtos com descontos</t>
         </is>
       </c>
-      <c r="E35" s="67" t="inlineStr">
+      <c r="E35" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -1974,34 +1997,34 @@
           <t>O Festas Válidas, até dia onze, no Antunes Mais. As melhores lojas de Catanduva, reunidas em um único lugar, com até setenta por cento off. Você já sabe de qual evento estamos falando? Bazar chique, é</t>
         </is>
       </c>
-      <c r="G35" s="67" t="inlineStr">
+      <c r="G35" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Antunes_Mais__Produtos_com_descontos__09-03-2026_09-06-15__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="67" t="inlineStr">
+      <c r="A36" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:06:15</t>
         </is>
       </c>
-      <c r="B36" s="67" t="inlineStr">
+      <c r="B36" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C36" s="67" t="inlineStr">
+      <c r="C36" s="72" t="inlineStr">
         <is>
           <t>Bazar Chique</t>
         </is>
       </c>
-      <c r="D36" s="67" t="inlineStr">
+      <c r="D36" s="72" t="inlineStr">
         <is>
           <t>Roupas, acessórios, calçados, óticas</t>
         </is>
       </c>
-      <c r="E36" s="67" t="inlineStr">
+      <c r="E36" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2011,34 +2034,34 @@
           <t>O Festas Válidas, até dia onze, no Antunes Mais. As melhores lojas de Catanduva, reunidas em um único lugar, com até setenta por cento off. Você já sabe de qual evento estamos falando? Bazar chique, é</t>
         </is>
       </c>
-      <c r="G36" s="67" t="inlineStr">
+      <c r="G36" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Bazar_Chique__Roupas__acessorios__calcados__oticas__09-03-2026_09-06-15__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="67" t="inlineStr">
+      <c r="A37" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:06:33</t>
         </is>
       </c>
-      <c r="B37" s="67" t="inlineStr">
+      <c r="B37" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C37" s="67" t="inlineStr">
+      <c r="C37" s="72" t="inlineStr">
         <is>
           <t>SimComércio e Vive Empre</t>
         </is>
       </c>
-      <c r="D37" s="67" t="inlineStr">
+      <c r="D37" s="72" t="inlineStr">
         <is>
           <t>Feira ou evento de vendas</t>
         </is>
       </c>
-      <c r="E37" s="67" t="inlineStr">
+      <c r="E37" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2048,34 +2071,34 @@
           <t>e muito mais com preços imperdíveis. Dias 19, 20 e 21 de março, na sede do SimComércio, Avenida Benedito Zancaner, 720, quinta e sexta, das nove às vinte e duas horas. Sábado, das nove às dezessete ho</t>
         </is>
       </c>
-      <c r="G37" s="67" t="inlineStr">
+      <c r="G37" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__SimComercio_e_Vive_Empre__Feira_ou_evento_de_vendas__09-03-2026_09-06-33.mp3</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="67" t="inlineStr">
+      <c r="A38" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:06:52</t>
         </is>
       </c>
-      <c r="B38" s="67" t="inlineStr">
+      <c r="B38" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C38" s="67" t="inlineStr">
+      <c r="C38" s="72" t="inlineStr">
         <is>
           <t>Vive Empreendimentos</t>
         </is>
       </c>
-      <c r="D38" s="67" t="inlineStr">
+      <c r="D38" s="72" t="inlineStr">
         <is>
           <t>empreendimentos imobiliários</t>
         </is>
       </c>
-      <c r="E38" s="67" t="inlineStr">
+      <c r="E38" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2085,34 +2108,34 @@
           <t>Olha, se tem uma empresa que vem transformando o jeito de viver dos últimos anos, essa empresa seguramente é a Vive Empreendimentos. Nascida em Catanduva, a Vive hoje está presente em quatro estados d</t>
         </is>
       </c>
-      <c r="G38" s="67" t="inlineStr">
+      <c r="G38" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Vive_Empreendimentos__empreendimentos_imobiliarios__09-03-2026_09-06-52.mp3</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="67" t="inlineStr">
+      <c r="A39" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:07:08</t>
         </is>
       </c>
-      <c r="B39" s="67" t="inlineStr">
+      <c r="B39" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C39" s="67" t="inlineStr">
+      <c r="C39" s="72" t="inlineStr">
         <is>
           <t>Vive</t>
         </is>
       </c>
-      <c r="D39" s="67" t="inlineStr">
+      <c r="D39" s="72" t="inlineStr">
         <is>
           <t>Loteamentos e espaços planejados</t>
         </is>
       </c>
-      <c r="E39" s="67" t="inlineStr">
+      <c r="E39" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2122,34 +2145,34 @@
           <t>Atenção, São Paulo, Mato Grosso do Sul, Minas Gerais e Goiás. Sempre levando desempenho com responsabilidade, sustentabilidade e muita inovação. Quem conhece os projetos da Vive sabe, não são apenas l</t>
         </is>
       </c>
-      <c r="G39" s="67" t="inlineStr">
+      <c r="G39" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Vive__Loteamentos_e_espacos_planejados__09-03-2026_09-07-08.mp3</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="67" t="inlineStr">
+      <c r="A40" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:07:26</t>
         </is>
       </c>
-      <c r="B40" s="67" t="inlineStr">
+      <c r="B40" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C40" s="67" t="inlineStr">
+      <c r="C40" s="72" t="inlineStr">
         <is>
           <t>VIB</t>
         </is>
       </c>
-      <c r="D40" s="67" t="inlineStr">
+      <c r="D40" s="72" t="inlineStr">
         <is>
           <t>empreendimentos imobiliários</t>
         </is>
       </c>
-      <c r="E40" s="67" t="inlineStr">
+      <c r="E40" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2159,34 +2182,34 @@
           <t>para oferecer mais qualidade de vida, contato com a natureza e toda a infraestrutura que as famílias procuram para viver bem. E tem mais, como coligada no grupo Serradinho, a VIB carrega a credibilida</t>
         </is>
       </c>
-      <c r="G40" s="67" t="inlineStr">
+      <c r="G40" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__VIB__empreendimentos_imobiliarios__09-03-2026_09-07-26.mp3</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="67" t="inlineStr">
+      <c r="A41" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:07:44</t>
         </is>
       </c>
-      <c r="B41" s="67" t="inlineStr">
+      <c r="B41" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C41" s="67" t="inlineStr">
+      <c r="C41" s="72" t="inlineStr">
         <is>
           <t>Oralfai Catanduva</t>
         </is>
       </c>
-      <c r="D41" s="67" t="inlineStr">
+      <c r="D41" s="72" t="inlineStr">
         <is>
           <t>tratamentos odontológicos</t>
         </is>
       </c>
-      <c r="E41" s="67" t="inlineStr">
+      <c r="E41" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2196,34 +2219,34 @@
           <t xml:space="preserve">Visão de futuro e compromisso com as cidades onde atua, vive empreendimentos conectando pessoas, criando novas formas de viver e mudando o futuro. Jovem Pan Olá, eu sou o doutor Guilherme Pelegrin da </t>
         </is>
       </c>
-      <c r="G41" s="67" t="inlineStr">
+      <c r="G41" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Oralfai_Catanduva__tratamentos_odontologicos__09-03-2026_09-07-44.mp3</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="67" t="inlineStr">
+      <c r="A42" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:08:38</t>
         </is>
       </c>
-      <c r="B42" s="67" t="inlineStr">
+      <c r="B42" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C42" s="67" t="inlineStr">
+      <c r="C42" s="72" t="inlineStr">
         <is>
           <t>Cacau Show</t>
         </is>
       </c>
-      <c r="D42" s="67" t="inlineStr">
+      <c r="D42" s="72" t="inlineStr">
         <is>
           <t>Ovos de Páscoa e tabletes</t>
         </is>
       </c>
-      <c r="E42" s="67" t="inlineStr">
+      <c r="E42" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2233,34 +2256,34 @@
           <t>E nos momentos em memórias que ficam para sempre. E quando o assunto é celebrar com sabor, a escolha é uma só. Cacau Show. Ovos de Páscoa encantadores. Tabletes irresistíveis. Presentes que emocionam.</t>
         </is>
       </c>
-      <c r="G42" s="67" t="inlineStr">
+      <c r="G42" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Cacau_Show__Ovos_de_Pascoa_e_tabletes__09-03-2026_09-08-38.mp3</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="67" t="inlineStr">
+      <c r="A43" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:09:51</t>
         </is>
       </c>
-      <c r="B43" s="67" t="inlineStr">
+      <c r="B43" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C43" s="67" t="inlineStr">
+      <c r="C43" s="72" t="inlineStr">
         <is>
           <t>Jovem Pan</t>
         </is>
       </c>
-      <c r="D43" s="67" t="inlineStr">
+      <c r="D43" s="72" t="inlineStr">
         <is>
           <t>Cobertura da Copa do Mundo</t>
         </is>
       </c>
-      <c r="E43" s="67" t="inlineStr">
+      <c r="E43" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2270,34 +2293,34 @@
           <t>Agora é dois mil e vinte e seis. Estados Unidos, México e Canadá. Desde sempre, a Jovem Pan está presente nas Copas do Mundo com equipe completa, informação em tempo real, opinião forte e a energia de</t>
         </is>
       </c>
-      <c r="G43" s="67" t="inlineStr">
+      <c r="G43" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Jovem_Pan__Cobertura_da_Copa_do_Mundo__09-03-2026_09-09-51.mp3</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="67" t="inlineStr">
+      <c r="A44" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:14:02</t>
         </is>
       </c>
-      <c r="B44" s="67" t="inlineStr">
+      <c r="B44" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C44" s="67" t="inlineStr">
+      <c r="C44" s="72" t="inlineStr">
         <is>
           <t>Cacau Show</t>
         </is>
       </c>
-      <c r="D44" s="67" t="inlineStr">
+      <c r="D44" s="72" t="inlineStr">
         <is>
           <t>Ovo de Páscoa</t>
         </is>
       </c>
-      <c r="E44" s="67" t="inlineStr">
+      <c r="E44" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2307,34 +2330,34 @@
           <t>porque ele tá dando mau exemplo do programa, eu acho que ele tá muito besteirento, ô Babu, você tá muito besteirento, Babu, para de falar, tá falando muita besteira e ainda tá causando esse alvoroço n</t>
         </is>
       </c>
-      <c r="G44" s="67" t="inlineStr">
+      <c r="G44" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Cacau_Show__Ovo_de_Pascoa__09-03-2026_09-14-02.mp3</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="67" t="inlineStr">
+      <c r="A45" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:14:20</t>
         </is>
       </c>
-      <c r="B45" s="67" t="inlineStr">
+      <c r="B45" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C45" s="67" t="inlineStr">
+      <c r="C45" s="72" t="inlineStr">
         <is>
           <t>Jovem Pan</t>
         </is>
       </c>
-      <c r="D45" s="67" t="inlineStr">
+      <c r="D45" s="72" t="inlineStr">
         <is>
           <t>Ovo de Páscoa Cacau Show</t>
         </is>
       </c>
-      <c r="E45" s="67" t="inlineStr">
+      <c r="E45" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2344,34 +2367,34 @@
           <t xml:space="preserve">E nas redes sociais, a hashtag tá lá, Babu Expulso, o que que cê acha? Conta aí que eu quero saber, no finalzinho, da hora do Manhã Pan. Fique ligado porque tem o ovo de páscoa cacau show, tá rolando </t>
         </is>
       </c>
-      <c r="G45" s="67" t="inlineStr">
+      <c r="G45" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__Jovem_Pan__Ovo_de_Pascoa_Cacau_Show__09-03-2026_09-14-20.mp3</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="67" t="inlineStr">
+      <c r="A46" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:14:24</t>
         </is>
       </c>
-      <c r="B46" s="67" t="inlineStr">
+      <c r="B46" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C46" s="67" t="inlineStr">
+      <c r="C46" s="72" t="inlineStr">
         <is>
           <t>Sotintas</t>
         </is>
       </c>
-      <c r="D46" s="67" t="inlineStr">
+      <c r="D46" s="72" t="inlineStr">
         <is>
           <t>loja de produtos</t>
         </is>
       </c>
-      <c r="E46" s="67" t="inlineStr">
+      <c r="E46" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2381,7 +2404,7 @@
           <t>Música Não saia daí, já já tem muito mais músicas aqui na Band FM Música Conheça a nova loja da Sotintas em Catanduva, na avenida Berendito Zancaner 1481 Um novo, moderno e amplo espaço para você conh</t>
         </is>
       </c>
-      <c r="G46" s="67" t="inlineStr">
+      <c r="G46" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Sotintas__loja_de_produtos__09-03-2026_09-14-24__ad1.mp3</t>
         </is>
@@ -2425,27 +2448,27 @@
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="67" t="inlineStr">
+      <c r="A48" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:15:00</t>
         </is>
       </c>
-      <c r="B48" s="67" t="inlineStr">
+      <c r="B48" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C48" s="67" t="inlineStr">
+      <c r="C48" s="72" t="inlineStr">
         <is>
           <t>Tatinho Veículos</t>
         </is>
       </c>
-      <c r="D48" s="67" t="inlineStr">
+      <c r="D48" s="72" t="inlineStr">
         <is>
           <t>Veículos</t>
         </is>
       </c>
-      <c r="E48" s="67" t="inlineStr">
+      <c r="E48" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2455,7 +2478,7 @@
           <t>José Nelson Machado, mil trezentos e setenta e nove, e agora também, na Avenida Benedito Zancanet, mil quatrocentos e oitenta e um, ao lado do Proença Supermercados. Só tintas, tudo em tintas, pra com</t>
         </is>
       </c>
-      <c r="G48" s="67" t="inlineStr">
+      <c r="G48" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Tatinho_Veiculos__Veiculos__09-03-2026_09-15-00.mp3</t>
         </is>
@@ -2499,27 +2522,27 @@
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="67" t="inlineStr">
+      <c r="A50" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:17:16</t>
         </is>
       </c>
-      <c r="B50" s="67" t="inlineStr">
+      <c r="B50" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C50" s="67" t="inlineStr">
+      <c r="C50" s="72" t="inlineStr">
         <is>
           <t>Alto Posto Campeão</t>
         </is>
       </c>
-      <c r="D50" s="67" t="inlineStr">
+      <c r="D50" s="72" t="inlineStr">
         <is>
           <t>Combustível</t>
         </is>
       </c>
-      <c r="E50" s="67" t="inlineStr">
+      <c r="E50" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2529,34 +2552,34 @@
           <t>Filos folha dupla, vinte metros, com doze unidades, doze e noventa e nove. Refrigerante, roler cola pet, dois litros, seis e noventa e nove. Procuro, mora, esquete, supermercados, qualidade, confiança</t>
         </is>
       </c>
-      <c r="G50" s="67" t="inlineStr">
+      <c r="G50" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Alto_Posto_Campeao__Combustivel__09-03-2026_09-17-16__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="67" t="inlineStr">
+      <c r="A51" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:17:33</t>
         </is>
       </c>
-      <c r="B51" s="67" t="inlineStr">
+      <c r="B51" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C51" s="67" t="inlineStr">
+      <c r="C51" s="72" t="inlineStr">
         <is>
           <t>Bande FM</t>
         </is>
       </c>
-      <c r="D51" s="67" t="inlineStr">
+      <c r="D51" s="72" t="inlineStr">
         <is>
           <t>Rádio</t>
         </is>
       </c>
-      <c r="E51" s="67" t="inlineStr">
+      <c r="E51" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2566,34 +2589,34 @@
           <t>É bem melhor, é Bande FM.</t>
         </is>
       </c>
-      <c r="G51" s="67" t="inlineStr">
+      <c r="G51" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Bande_FM__Radio__09-03-2026_09-17-33.mp3</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="67" t="inlineStr">
+      <c r="A52" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:30:51</t>
         </is>
       </c>
-      <c r="B52" s="67" t="inlineStr">
+      <c r="B52" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C52" s="67" t="inlineStr">
+      <c r="C52" s="72" t="inlineStr">
         <is>
           <t>Traia Veia</t>
         </is>
       </c>
-      <c r="D52" s="67" t="inlineStr">
+      <c r="D52" s="72" t="inlineStr">
         <is>
           <t>Evento (show)</t>
         </is>
       </c>
-      <c r="E52" s="67" t="inlineStr">
+      <c r="E52" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2603,7 +2626,7 @@
           <t>Primeira vez na região, Traia Veia! E em palco, 360! Mesas, open pool de open bar e convites para área VIP, a venda na Secretaria do Clube ou querodoisingressos.com.br Seu moço e Traia Veia! Dia 20 de</t>
         </is>
       </c>
-      <c r="G52" s="67" t="inlineStr">
+      <c r="G52" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Traia_Veia__Evento__show__09-03-2026_09-30-51__ad1.mp3</t>
         </is>
@@ -2647,27 +2670,27 @@
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="67" t="inlineStr">
+      <c r="A54" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:30:51</t>
         </is>
       </c>
-      <c r="B54" s="67" t="inlineStr">
+      <c r="B54" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C54" s="67" t="inlineStr">
+      <c r="C54" s="72" t="inlineStr">
         <is>
           <t>Quero Dois Ingressos</t>
         </is>
       </c>
-      <c r="D54" s="67" t="inlineStr">
+      <c r="D54" s="72" t="inlineStr">
         <is>
           <t>Serviço de venda de ingressos</t>
         </is>
       </c>
-      <c r="E54" s="67" t="inlineStr">
+      <c r="E54" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2677,34 +2700,34 @@
           <t>Primeira vez na região, Traia Veia! E em palco, 360! Mesas, open pool de open bar e convites para área VIP, a venda na Secretaria do Clube ou querodoisingressos.com.br Seu moço e Traia Veia! Dia 20 de</t>
         </is>
       </c>
-      <c r="G54" s="67" t="inlineStr">
+      <c r="G54" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Quero_Dois_Ingressos__Servico_de_venda_de_ingressos__09-03-2026_09-30-51__ad3.mp3</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="67" t="inlineStr">
+      <c r="A55" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:31:07</t>
         </is>
       </c>
-      <c r="B55" s="67" t="inlineStr">
+      <c r="B55" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C55" s="67" t="inlineStr">
+      <c r="C55" s="72" t="inlineStr">
         <is>
           <t>Clube de Tênis Catanduva</t>
         </is>
       </c>
-      <c r="D55" s="67" t="inlineStr">
+      <c r="D55" s="72" t="inlineStr">
         <is>
           <t>Ingressos</t>
         </is>
       </c>
-      <c r="E55" s="67" t="inlineStr">
+      <c r="E55" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2714,34 +2737,34 @@
           <t>A venda na Secretaria do Clube ou quero dois ingressos ponto com ponto BR. Seu moço e praia velha, dia vinte de março no Clube de Tênis Catanduva. Na vida, os imprevistos são comuns. Aquela viagem ine</t>
         </is>
       </c>
-      <c r="G55" s="67" t="inlineStr">
+      <c r="G55" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Clube_de_Tenis_Catanduva__Ingressos__09-03-2026_09-31-07.mp3</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="67" t="inlineStr">
+      <c r="A56" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:31:56</t>
         </is>
       </c>
-      <c r="B56" s="67" t="inlineStr">
+      <c r="B56" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C56" s="67" t="inlineStr">
+      <c r="C56" s="72" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="D56" s="67" t="inlineStr">
+      <c r="D56" s="72" t="inlineStr">
         <is>
           <t>Produtos alimentícios (peixe, camarão, farinha, queijo, papel)</t>
         </is>
       </c>
-      <c r="E56" s="67" t="inlineStr">
+      <c r="E56" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2751,34 +2774,34 @@
           <t>Peixe e muito mais, tudo com preço baixinho pra você aproveitar. Filé de peito laro, 1,1497. Camarão palimara, 180 gramas, 1,1497. Farinha globo, 1,247. Tó de 370 gramas, 7,99. Mussarela a partir de 2</t>
         </is>
       </c>
-      <c r="G56" s="67" t="inlineStr">
+      <c r="G56" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Mar__Produtos_alimenticios__peixe__camarao__farinha__queijo__pape__09-03-2026_09-31-56.mp3</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="67" t="inlineStr">
+      <c r="A57" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:32:13</t>
         </is>
       </c>
-      <c r="B57" s="67" t="inlineStr">
+      <c r="B57" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C57" s="67" t="inlineStr">
+      <c r="C57" s="72" t="inlineStr">
         <is>
           <t>Atacarejo Mar</t>
         </is>
       </c>
-      <c r="D57" s="67" t="inlineStr">
+      <c r="D57" s="72" t="inlineStr">
         <is>
           <t>Páscoa</t>
         </is>
       </c>
-      <c r="E57" s="67" t="inlineStr">
+      <c r="E57" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2788,7 +2811,7 @@
           <t xml:space="preserve">Tocando Papel Supra, vinte e nove e noventa. A maior páscoa do atacarejo é no mar. De voltar aqui na Ondas Verdes, nove e trinta e um agora. Alô, Toninha, bom dia, cê tá boa? Eu sou bem abençoado pra </t>
         </is>
       </c>
-      <c r="G57" s="67" t="inlineStr">
+      <c r="G57" s="72" t="inlineStr">
         <is>
           <t>Ondas_Verdes__Atacarejo_Mar__Pascoa__09-03-2026_09-32-13.mp3</t>
         </is>
@@ -2869,27 +2892,27 @@
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="67" t="inlineStr">
+      <c r="A60" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:35:56</t>
         </is>
       </c>
-      <c r="B60" s="67" t="inlineStr">
+      <c r="B60" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C60" s="67" t="inlineStr">
+      <c r="C60" s="72" t="inlineStr">
         <is>
           <t>Rede Móveis Casa Vende</t>
         </is>
       </c>
-      <c r="D60" s="67" t="inlineStr">
+      <c r="D60" s="72" t="inlineStr">
         <is>
           <t>Produtos para renovar a casa</t>
         </is>
       </c>
-      <c r="E60" s="67" t="inlineStr">
+      <c r="E60" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2899,34 +2922,34 @@
           <t>Não saia daí, já já tem muito mais músicas aqui na Band FM. Band FM Atenção Catanduva e região, é aniversário da Rede Móveis Casa Vende. Com ofertas especiais para renovar a sua casa. Produtos selecio</t>
         </is>
       </c>
-      <c r="G60" s="67" t="inlineStr">
+      <c r="G60" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Rede_Moveis_Casa_Vende__Produtos_para_renovar_a_casa__09-03-2026_09-35-56.mp3</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="67" t="inlineStr">
+      <c r="A61" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:36:33</t>
         </is>
       </c>
-      <c r="B61" s="67" t="inlineStr">
+      <c r="B61" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C61" s="67" t="inlineStr">
+      <c r="C61" s="72" t="inlineStr">
         <is>
           <t>Cressol</t>
         </is>
       </c>
-      <c r="D61" s="67" t="inlineStr">
+      <c r="D61" s="72" t="inlineStr">
         <is>
           <t>Promoção Operar é Ganhar</t>
         </is>
       </c>
-      <c r="E61" s="67" t="inlineStr">
+      <c r="E61" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2936,34 +2959,34 @@
           <t xml:space="preserve">Dá pra contar com a sorte, né? Mas se a sorte te ajudar, você ainda pode ganhar 12 milhões em prêmios com a promoção Operar é Ganhar. Invista com a Cressol, gere números da sorte e concorra. Você vai </t>
         </is>
       </c>
-      <c r="G61" s="67" t="inlineStr">
+      <c r="G61" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Cressol__Promocao_Operar_e_Ganhar__09-03-2026_09-36-33__ad1.mp3</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="67" t="inlineStr">
+      <c r="A62" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:36:33</t>
         </is>
       </c>
-      <c r="B62" s="67" t="inlineStr">
+      <c r="B62" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C62" s="67" t="inlineStr">
+      <c r="C62" s="72" t="inlineStr">
         <is>
           <t>Alto Posto Campeão</t>
         </is>
       </c>
-      <c r="D62" s="67" t="inlineStr">
+      <c r="D62" s="72" t="inlineStr">
         <is>
           <t>Combustível</t>
         </is>
       </c>
-      <c r="E62" s="67" t="inlineStr">
+      <c r="E62" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -2973,34 +2996,34 @@
           <t xml:space="preserve">Dá pra contar com a sorte, né? Mas se a sorte te ajudar, você ainda pode ganhar 12 milhões em prêmios com a promoção Operar é Ganhar. Invista com a Cressol, gere números da sorte e concorra. Você vai </t>
         </is>
       </c>
-      <c r="G62" s="67" t="inlineStr">
+      <c r="G62" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Alto_Posto_Campeao__Combustivel__09-03-2026_09-36-33__ad2.mp3</t>
         </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="67" t="inlineStr">
+      <c r="A63" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:36:50</t>
         </is>
       </c>
-      <c r="B63" s="67" t="inlineStr">
+      <c r="B63" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C63" s="67" t="inlineStr">
+      <c r="C63" s="72" t="inlineStr">
         <is>
           <t>Alto Posto Campeão</t>
         </is>
       </c>
-      <c r="D63" s="67" t="inlineStr">
+      <c r="D63" s="72" t="inlineStr">
         <is>
           <t>Combustível e conveniência</t>
         </is>
       </c>
-      <c r="E63" s="67" t="inlineStr">
+      <c r="E63" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -3010,34 +3033,34 @@
           <t>Só poderá é ganhar Certificado de autorização SPAME, número 04047374 Alto Posto Campeão, o seu destino de qualidade em combustível Vá conhecer o Alto Posto Campeão, onde qualidade e preço campeão anda</t>
         </is>
       </c>
-      <c r="G63" s="67" t="inlineStr">
+      <c r="G63" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Alto_Posto_Campeao__Combustivel_e_conveniencia__09-03-2026_09-36-50.mp3</t>
         </is>
       </c>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="67" t="inlineStr">
+      <c r="A64" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:37:08</t>
         </is>
       </c>
-      <c r="B64" s="67" t="inlineStr">
+      <c r="B64" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan</t>
         </is>
       </c>
-      <c r="C64" s="67" t="inlineStr">
+      <c r="C64" s="72" t="inlineStr">
         <is>
           <t>UOL</t>
         </is>
       </c>
-      <c r="D64" s="67" t="inlineStr">
+      <c r="D64" s="72" t="inlineStr">
         <is>
           <t>Enquete do Big Brother 26</t>
         </is>
       </c>
-      <c r="E64" s="67" t="inlineStr">
+      <c r="E64" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -3047,34 +3070,34 @@
           <t>Rafa, que negócio do Babu, hein? Babu, eu vou te falar, hein, Babu? O Paulo mandou pra gente aqui, o nosso ouvinte, ele falou assim Ô Rafa, cola no site do UOL Vai lá no UOL que tem a enquete A enquet</t>
         </is>
       </c>
-      <c r="G64" s="67" t="inlineStr">
+      <c r="G64" s="72" t="inlineStr">
         <is>
           <t>Jovem_Pan__UOL__Enquete_do_Big_Brother_26__09-03-2026_09-37-08.mp3</t>
         </is>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="68" t="inlineStr">
+      <c r="A65" s="72" t="inlineStr">
         <is>
           <t>09/03/2026 09:39:48</t>
         </is>
       </c>
-      <c r="B65" s="68" t="inlineStr">
+      <c r="B65" s="72" t="inlineStr">
         <is>
           <t>Band_FM</t>
         </is>
       </c>
-      <c r="C65" s="68" t="inlineStr">
+      <c r="C65" s="72" t="inlineStr">
         <is>
           <t>Grupo Moresque</t>
         </is>
       </c>
-      <c r="D65" s="68" t="inlineStr">
+      <c r="D65" s="72" t="inlineStr">
         <is>
           <t>Carnes e arroz</t>
         </is>
       </c>
-      <c r="E65" s="68" t="inlineStr">
+      <c r="E65" s="72" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
@@ -3084,9 +3107,194 @@
           <t>o mundo. Atenção para algumas das grandes ofertas do Grupo Moresque válidas até dia nove de março. Alcatra com a minha bovina quilo quarenta e três e noventa e nove contra filé bovino quilo quarenta e</t>
         </is>
       </c>
-      <c r="G65" s="68" t="inlineStr">
+      <c r="G65" s="72" t="inlineStr">
         <is>
           <t>Band_FM__Grupo_Moresque__Carnes_e_arroz__09-03-2026_09-39-48.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="73" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:03:52</t>
+        </is>
+      </c>
+      <c r="B66" s="73" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes</t>
+        </is>
+      </c>
+      <c r="C66" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D66" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="73" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="F66" s="70" t="inlineStr">
+        <is>
+          <t>Primeiro par de lentes multifocais digitais da linha Nobre com antirreflexo, o segundo par é grátis. Consulte condições na loja, tá? E tem muito mais. Lentes de visão simples com antirreflexo e filtro</t>
+        </is>
+      </c>
+      <c r="G66" s="73" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Desconhecido__09-03-2026_10-03-52.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="72" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:05:17</t>
+        </is>
+      </c>
+      <c r="B67" s="72" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C67" s="72" t="inlineStr">
+        <is>
+          <t>Band FM</t>
+        </is>
+      </c>
+      <c r="D67" s="72" t="inlineStr">
+        <is>
+          <t>Rádio/Programa</t>
+        </is>
+      </c>
+      <c r="E67" s="72" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lógico, comentar nas nossas redes sociais. É isso que eu tava pensando. Escolher o nome e ganhar o mascote mais gostosinho do rádio brasileiro. É tudo de bom. É tudo de Band. Band FM. Band FM. Queria </t>
+        </is>
+      </c>
+      <c r="G67" s="72" t="inlineStr">
+        <is>
+          <t>Band_FM__Band_FM__Radio_Programa__09-03-2026_10-05-17.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="72" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28:54</t>
+        </is>
+      </c>
+      <c r="B68" s="72" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C68" s="72" t="inlineStr">
+        <is>
+          <t>Band FM</t>
+        </is>
+      </c>
+      <c r="D68" s="72" t="inlineStr">
+        <is>
+          <t>Smartphone novo</t>
+        </is>
+      </c>
+      <c r="E68" s="72" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Vinte e seis, resolvendo a vida. É, tudo da Band é ótimo, né? Tudo de boa qualidade. Mande um WhatsApp pra Band FM dizendo Smartphone novo, é na Band FM. Pronto, já tá concorrendo. Vende presente toda</t>
+        </is>
+      </c>
+      <c r="G68" s="72" t="inlineStr">
+        <is>
+          <t>Band_FM__Band_FM__Smartphone_novo__09-03-2026_10-28-54.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="73" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:32:17</t>
+        </is>
+      </c>
+      <c r="B69" s="73" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C69" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D69" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="73" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="F69" s="70" t="inlineStr">
+        <is>
+          <t>Seu Moço, na abertura! E pela primeira vez na região, Traia Veia! Você só vai achar lembrança boa! E em palco 360! E o sinal abria! Convites para a área VIP por 80 reais, a venda na Secretaria do Club</t>
+        </is>
+      </c>
+      <c r="G69" s="73" t="inlineStr">
+        <is>
+          <t>Band_FM__Desconhecido__09-03-2026_10-32-17.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="74" t="inlineStr">
+        <is>
+          <t>09/03/2026 11:03:50</t>
+        </is>
+      </c>
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes</t>
+        </is>
+      </c>
+      <c r="C70" s="74" t="inlineStr">
+        <is>
+          <t>Ótica Fabrilein</t>
+        </is>
+      </c>
+      <c r="D70" s="74" t="inlineStr">
+        <is>
+          <t>Lentes e atendimento óptico</t>
+        </is>
+      </c>
+      <c r="E70" s="74" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Ah, ofertas válidas até dia vinte e dois de março ou enquanto durarem os estoques. Vem conferir, um a noventa e nove, quem economiza pode mais. Quando o assunto é visão, a ótica Fabrilein é referência</t>
+        </is>
+      </c>
+      <c r="G70" s="74" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Otica_Fabrilein__Lentes_e_atendimento_optico__09-03-2026_11-03-50.mp3</t>
         </is>
       </c>
     </row>
@@ -3128,11 +3336,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>09/03/2026 09:32:13</t>
+          <t>09/03/2026 11:03:50</t>
         </is>
       </c>
     </row>
@@ -3158,11 +3366,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>09/03/2026 09:39:48</t>
+          <t>09/03/2026 10:32:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update relatorio_anuncios.xlsx with new data and analysis
</commit_message>
<xml_diff>
--- a/radio_capture/relatorio_anuncios.xlsx
+++ b/radio_capture/relatorio_anuncios.xlsx
@@ -61,12 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -122,25 +122,55 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -508,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -520,7 +550,7 @@
     <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="60" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Data/Hora</t>
@@ -548,7 +578,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Transcrição (resumo)</t>
+          <t>Trecho do Anúncio</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -558,335 +588,705 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:11:29</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 09:42:25</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>Rede Móveis</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Rede Móveis Casa Vende</t>
+        </is>
+      </c>
+      <c r="G2" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Rede_Moveis__20-03-2026_09-42-24__ad1.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>20/03/2026 09:42:25</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>JS Consórcios</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Grupo JS Consórcios</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Band_FM__JS_Consorcios__20-03-2026_09-42-25__ad2.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 09:42:25</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Cressol Gele</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>números da sorte</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Cressol Gele números da sorte</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Cressol_Gele__numeros_da_sorte__20-03-2026_09-42-25__ad3.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>20/03/2026 09:43:12</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Cressol</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>promoção, prêmios, investimento</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Invista com a Cressol, gere números da sorte e concorra</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Band_FM__Cressol__promocao__premios__investimento__20-03-2026_09-43-12__ad1.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>20/03/2026 09:43:12</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>internet, suporte técnico, velocidade</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>A melhor internet da região é Netflix</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Band_FM__Netflix__internet__suporte_tecnico__velocidade__20-03-2026_09-43-12__ad2.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:03:19</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Grupo Moresc</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>refrigerante, sorvete, creme, piquenique, pet, vestidos de noiva</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Ofertas válidas até o dia vinte e três, nas lojas do Grupo Moresc</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Grupo_Moresc__refrigerante__sorvete__creme__piquenique__pet__vestidos_de_n__20-03-2026_10-03-19.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:04:07</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Dicopel</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>formas para ovos, bombons de acetato e silicone, embalagens, envelopes, caixa para ovos, papéis decorados, chocolates confeitos, linha completa de doces</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>A sua Páscoa é mais gostosa na Dicopel</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Dicopel__formas_para_ovos__bombons_de_acetato_e_silicone__embalagens___20-03-2026_10-04-07.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:04:48</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Top Frios</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>produtos exclusivos</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Produtos exclusivos, os menores preços, conforto pra você comprar e ainda, claro, estacionamento próprio. Top Frios é demais. Entregamos em domicílio. WhatsApp 997459897 ou 35239820. Top Frios, Rua 15</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes__Top_Frios__produtos_exclusivos__18-03-2026_15-11-29.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:11:46</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Desconhecido__20-03-2026_10-04-48.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:04:54</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>La Juma</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>apartamento, Ilhas Gregas, Rua Sergipe, três dormitórios, suíte, salas, cozinha</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Apartamento no edifício Ilhas Gregas</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__La_Juma__apartamento__Ilhas_Gregas__Rua_Sergipe__tres_dormitorios__su__20-03-2026_10-04-54.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:32:47</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Sicredi</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>poupança premiada</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Sicredi, poucos, é premiada</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Sicredi__poupanca_premiada__20-03-2026_10-32-47.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:33:35</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Padre Albino Saúde</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>serviços de saúde, profissionais de saúde</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>No Padre Albino Saúde</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Padre_Albino_Saude__servicos_de_saude__profissionais_de_saude__20-03-2026_10-33-35__ad1.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:33:35</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Paz Previme</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>serviços de saúde, profissionais de saúde</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>contando em breve com o novo prédio do Paz Previme</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Paz_Previme__servicos_de_saude__profissionais_de_saude__20-03-2026_10-33-35__ad2.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:34:23</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Rede Móveis Casa Verde</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>produtos selecionados</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>ofertas especiais pra renovar a sua casa</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Rede_Moveis_Casa_Verde__produtos_selecionados__20-03-2026_10-34-23__ad1.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:34:23</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Cressol</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>investimento, prêmios</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Invista com a Cressol Gere números da sorte e concorra</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>Band_FM__Cressol__investimento__premios__20-03-2026_10-34-23__ad2.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:36:36</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>vestido de noiva</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 98, 20, top frios, rua 15 de novembro, 1306, com estacionamento próprio. Você que vai casar, pare um instante. Imagine encontrar um vestido de noiva, maravilhoso, por apenas 200 reais. Sim, 2</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes__Desconhecido__vestido_de_noiva__18-03-2026_15-11-46.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:12:02</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Ferreira Decorações</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>tapete, cortinas</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Ferreira Decorações, uma verdadeira festa</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Ferreira_Decoracoes__tapete__cortinas__20-03-2026_10-36-36.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:53:39</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>bazar de vestidos de noiva</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Maravilhoso, por apenas duzentos reais. Sim, duzentos reais. No dia vinte e oito de março, sábado, a partir das dez horas da manhã, acontece o grande bazar de vestidos de noiva em prol do projeto Coru</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes__Desconhecido__bazar_de_vestidos_de_noiva__18-03-2026_15-12-02.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:12:19</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>Vance Brasil</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>ofertas, cerveja Romarinho, Antártica, Escoa, Brama</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Cerveja Romarinho, Antártica, Escoa e Brama, dois e quarenta e nove</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Vance_Brasil__ofertas__cerveja_Romarinho__Antartica__Escoa__Brama__20-03-2026_10-53-39.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:55:13</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Messias Doces</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>ovos de Páscoa</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Serão mais de oitenta vestidos de noiva, lindos, esperando você. Rua São Paulo, mil e trinta e três, sábado, dia vinte e oito, a partir das dez da manhã. Informações WhatsApp, dezessete, nove dois, ze</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes__Messias_Doces__ovos_de_Pascoa__18-03-2026_15-12-19.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:13:58</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Empório São Pedro</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>bacalhau selecionado, azeites especiais, azeitonas e grão de bico premium</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Empório São Pedro, bacalhau selecionado, azeites especiais, azeitonas e grão de </t>
+        </is>
+      </c>
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Emporio_Sao_Pedro__bacalhau_selecionado__azeites_especiais__azeitonas_e_grao_de__20-03-2026_10-55-13__ad1.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:55:13</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>Ondas_Verdes</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Polo São Pedro</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>bacalhau de qualidade</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>de Catanduva. Bacalhau de qualidade, com procedência e aquele cuidado especial. Venha garantir o seu, na Rua São Paulo, cinquenta e quatro. Em Polo São Pedro, tradição que dá sabor a sua mesa. Canecão</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes__Polo_Sao_Pedro__bacalhau_de_qualidade__18-03-2026_15-13-58__ad1.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:13:58</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>carro ou caminhonete</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>de Catanduva. Bacalhau de qualidade, com procedência e aquele cuidado especial. Venha garantir o seu, na Rua São Paulo, cinquenta e quatro. Em Polo São Pedro, tradição que dá sabor a sua mesa. Canecão</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Ondas_Verdes__Desconhecido__carro_ou_caminhonete__18-03-2026_15-13-58__ad2.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:14:45</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Band_FM</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>Magazine Luiza</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>iPhone</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>É isso mesmo, ó. Vem comprar o seu iPhone aqui no Magazine Luiza em 21 vezes sem juros. Temos também o Galaxy S25, 256 GB por apenas 3.999. Também, Maurício, em 21 vezes sem juros no cartão do Magazin</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Band_FM__Magazine_Luiza__iPhone__18-03-2026_15-14-45.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:15:51</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Band_FM</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Magazine Luiza</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>cartão</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Hein, Maurício? Em 21 vezes sem juros no cartão do Magazine Luiza. Temos Motorola também na promoção aqui, Motorola, Edge 60, Fusio, 256 gigas, por apenas 299 ou 21 pagamentos sem juros no cartão do M</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>Band_FM__Magazine_Luiza__cartao__18-03-2026_15-15-51__ad1.mp3</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>18/03/2026 15:15:51</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Band_FM</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Motorola</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Edge 60, Fusio</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Hein, Maurício? Em 21 vezes sem juros no cartão do Magazine Luiza. Temos Motorola também na promoção aqui, Motorola, Edge 60, Fusio, 256 gigas, por apenas 299 ou 21 pagamentos sem juros no cartão do M</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Band_FM__Motorola__Edge_60__Fusio__18-03-2026_15-15-51__ad2.mp3</t>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Óticas Fabrilene</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>lentes multifocais digitais Noblem com antirreflexo, lentes de visão simples com antirreflexo e filtro de luz azul</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Na compra do primeiro par de lentes multifocais digitais Noblem com antirreflexo</t>
+        </is>
+      </c>
+      <c r="G19" s="22" t="inlineStr">
+        <is>
+          <t>Ondas_Verdes__Oticas_Fabrilene__lentes_multifocais_digitais_Noblem_com_antirreflexo__lentes___20-03-2026_10-55-13__ad2.mp3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>20/03/2026 10:56:39</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Band_FM</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>Grupo Moresc</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>carne bovina, suína, frango, arroz, banana, leite</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>A 100 bovino, quilo 32,99. Mistéca suína, 14,99 o quilo.</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>Band_FM__Grupo_Moresc__carne_bovina__suina__frango__arroz__banana__leite__20-03-2026_10-56-39.mp3</t>
         </is>
       </c>
     </row>
@@ -924,30 +1324,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ondas_Verdes</t>
+          <t>Band_FM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>18/03/2026 15:13:58</t>
+          <t>20/03/2026 10:56:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Band_FM</t>
+          <t>Ondas_Verdes</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>18/03/2026 15:15:51</t>
+          <t>20/03/2026 10:55:13</t>
         </is>
       </c>
     </row>

</xml_diff>